<commit_message>
Added pooled water as a typology
</commit_message>
<xml_diff>
--- a/Copper/6. Statistical data analysis/Multiple linear regression/MLR.xlsx
+++ b/Copper/6. Statistical data analysis/Multiple linear regression/MLR.xlsx
@@ -40,12 +40,12 @@
     <t xml:space="preserve">log_DOC_nM_std</t>
   </si>
   <si>
+    <t xml:space="preserve">log_K_nM_std</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_Na_nM_std</t>
   </si>
   <si>
-    <t xml:space="preserve">log_K_nM_std</t>
-  </si>
-  <si>
     <t xml:space="preserve">log_SO4_nM_std</t>
   </si>
   <si>
@@ -55,13 +55,13 @@
     <t xml:space="preserve">log_Ca_nM_std</t>
   </si>
   <si>
+    <t xml:space="preserve">log_DIC_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Mg_nM_std</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_Temp_C_std</t>
-  </si>
-  <si>
-    <t xml:space="preserve">log_DIC_nM_std</t>
-  </si>
-  <si>
-    <t xml:space="preserve">log_Mg_nM_std</t>
   </si>
   <si>
     <t xml:space="preserve">Std. Error</t>
@@ -448,16 +448,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="n">
-        <v>1.34720729087859</v>
+        <v>1.35672869104225</v>
       </c>
       <c r="C2" t="n">
-        <v>1.93382755337073e-312</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>2.54560775861302</v>
+        <v>2.53871349901583</v>
       </c>
       <c r="E2" t="n">
-        <v>0.627087283938181</v>
+        <v>0.624230275778126</v>
       </c>
     </row>
     <row r="3">
@@ -465,16 +465,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.53074332141694</v>
+        <v>-0.555475496523478</v>
       </c>
       <c r="C3" t="n">
-        <v>7.88771978470265e-219</v>
+        <v>2.34738776024147e-246</v>
       </c>
       <c r="D3" t="n">
-        <v>1.44064520760624</v>
+        <v>1.39372800204517</v>
       </c>
       <c r="E3" t="n">
-        <v>0.147820642405235</v>
+        <v>0.156780509182818</v>
       </c>
     </row>
     <row r="4">
@@ -482,16 +482,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.655259618119645</v>
+        <v>-0.681355511740908</v>
       </c>
       <c r="C4" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000780422424244998</v>
+        <v>1.58959967639677e-219</v>
       </c>
       <c r="D4" t="n">
-        <v>2.79835401362034</v>
+        <v>2.97837008122367</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0906589436958603</v>
+        <v>0.0903126865969564</v>
       </c>
     </row>
     <row r="5">
@@ -499,16 +499,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.0026221572434501</v>
+        <v>-0.0120258168636827</v>
       </c>
       <c r="C5" t="n">
-        <v>0.917504985883087</v>
+        <v>0.276842504152492</v>
       </c>
       <c r="D5" t="n">
-        <v>19.3699009872279</v>
+        <v>3.96317191586794</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0290517929260689</v>
+        <v>0.0285220139759224</v>
       </c>
     </row>
     <row r="6">
@@ -516,16 +516,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.0120736553164605</v>
+        <v>-0.00569374207398377</v>
       </c>
       <c r="C6" t="n">
-        <v>0.345758948602271</v>
+        <v>0.798467787629099</v>
       </c>
       <c r="D6" t="n">
-        <v>4.94967528991723</v>
+        <v>16.1385210522413</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0285636618933346</v>
+        <v>0.024553492024105</v>
       </c>
     </row>
     <row r="7">
@@ -533,16 +533,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="n">
-        <v>0.032441084846519</v>
+        <v>0.0409257488241372</v>
       </c>
       <c r="C7" t="n">
-        <v>0.00557440539491165</v>
+        <v>0.000203955563127836</v>
       </c>
       <c r="D7" t="n">
-        <v>4.0939287415833</v>
+        <v>3.86868246299033</v>
       </c>
       <c r="E7" t="n">
-        <v>0.024317369731219</v>
+        <v>0.0239036932751181</v>
       </c>
     </row>
     <row r="8">
@@ -550,16 +550,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.034214480669279</v>
+        <v>-0.0471901271660138</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0648337866635752</v>
+        <v>0.00612154298784395</v>
       </c>
       <c r="D8" t="n">
-        <v>10.3265365918509</v>
+        <v>9.52265199934725</v>
       </c>
       <c r="E8" t="n">
-        <v>0.018892922623952</v>
+        <v>0.0166933827180247</v>
       </c>
     </row>
     <row r="9">
@@ -567,16 +567,16 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.0295168823648154</v>
+        <v>-0.0237065716067035</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0844451331890632</v>
+        <v>0.158161447835326</v>
       </c>
       <c r="D9" t="n">
-        <v>8.80630321544478</v>
+        <v>9.13404853479142</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0110393607655796</v>
+        <v>0.0129797927329226</v>
       </c>
     </row>
     <row r="10">
@@ -584,16 +584,16 @@
         <v>13</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.0552551142818269</v>
+        <v>-0.0140980592137172</v>
       </c>
       <c r="C10" t="n">
-        <v>0.000000000000000250562692550019</v>
+        <v>0.391164791926459</v>
       </c>
       <c r="D10" t="n">
-        <v>1.24409781629897</v>
+        <v>8.76450933834822</v>
       </c>
       <c r="E10" t="n">
-        <v>0.00941936334920962</v>
+        <v>0.00809406270159193</v>
       </c>
     </row>
     <row r="11">
@@ -601,16 +601,16 @@
         <v>14</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.0013580035556857</v>
+        <v>-0.0130572849002888</v>
       </c>
       <c r="C11" t="n">
-        <v>0.935259212217569</v>
+        <v>0.284720775809009</v>
       </c>
       <c r="D11" t="n">
-        <v>8.44716511552504</v>
+        <v>4.8280028331817</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00668730036121604</v>
+        <v>0.00766965920374788</v>
       </c>
     </row>
     <row r="12">
@@ -618,16 +618,16 @@
         <v>15</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.0288792080868142</v>
+        <v>-0.051092098784436</v>
       </c>
       <c r="C12" t="n">
-        <v>0.020075592105186</v>
+        <v>0.000000000000000779520063978463</v>
       </c>
       <c r="D12" t="n">
-        <v>4.62672094846105</v>
+        <v>1.19495270731042</v>
       </c>
       <c r="E12" t="n">
-        <v>0.00646135831014396</v>
+        <v>0.00626043181066737</v>
       </c>
     </row>
   </sheetData>
@@ -663,16 +663,16 @@
         <v>19</v>
       </c>
       <c r="B2" t="n">
-        <v>0.000000000000000494187339045713</v>
+        <v>-0.000000000000000509649550108252</v>
       </c>
       <c r="C2" t="n">
-        <v>0.00573986370212581</v>
+        <v>0.00553975506363742</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0000000000000860973996408113</v>
+        <v>-0.0000000000000919985711017365</v>
       </c>
       <c r="E2" t="n">
-        <v>0.999999999999931</v>
+        <v>0.999999999999927</v>
       </c>
     </row>
     <row r="3">
@@ -680,33 +680,33 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>1.34720729087859</v>
+        <v>1.35672869104225</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0091708194900048</v>
+        <v>0.00883813634006643</v>
       </c>
       <c r="D3" t="n">
-        <v>146.901516527165</v>
+        <v>153.508459118436</v>
       </c>
       <c r="E3" t="n">
-        <v>1.93382755337073e-312</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0552551142818269</v>
+        <v>-0.051092098784436</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0064112050354191</v>
+        <v>0.00606358136349781</v>
       </c>
       <c r="D4" t="n">
-        <v>-8.61852241139796</v>
+        <v>-8.42605973624856</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000000000000000250562692550019</v>
+        <v>0.000000000000000779520063978463</v>
       </c>
     </row>
     <row r="5">
@@ -714,16 +714,16 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.53074332141694</v>
+        <v>-0.555475496523478</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00689907588208905</v>
+        <v>0.00654851555696949</v>
       </c>
       <c r="D5" t="n">
-        <v>-76.9296251393353</v>
+        <v>-84.8246433395572</v>
       </c>
       <c r="E5" t="n">
-        <v>7.88771978470265e-219</v>
+        <v>2.34738776024147e-246</v>
       </c>
     </row>
     <row r="6">
@@ -731,33 +731,33 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.655259618119645</v>
+        <v>-0.681355511740908</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00961531972760117</v>
+        <v>0.0095728924786171</v>
       </c>
       <c r="D6" t="n">
-        <v>-68.1474601659574</v>
+        <v>-71.175510773034</v>
       </c>
       <c r="E6" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000780422424244998</v>
+        <v>1.58959967639677e-219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.0013580035556857</v>
+        <v>-0.0140980592137172</v>
       </c>
       <c r="C7" t="n">
-        <v>0.016705823702953</v>
+        <v>0.0164216826367651</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0812892306199575</v>
+        <v>-0.858502720187414</v>
       </c>
       <c r="E7" t="n">
-        <v>0.935259212217569</v>
+        <v>0.391164791926459</v>
       </c>
     </row>
     <row r="8">
@@ -765,16 +765,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.034214480669279</v>
+        <v>-0.0471901271660138</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0184709718498691</v>
+        <v>0.0171172032484941</v>
       </c>
       <c r="D8" t="n">
-        <v>-1.85233787086961</v>
+        <v>-2.75688303053627</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0648337866635752</v>
+        <v>0.00612154298784395</v>
       </c>
     </row>
     <row r="9">
@@ -782,33 +782,33 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.0295168823648154</v>
+        <v>-0.0237065716067035</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0170572580502615</v>
+        <v>0.0167643032494583</v>
       </c>
       <c r="D9" t="n">
-        <v>-1.73045880397892</v>
+        <v>-1.41411016335972</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0844451331890632</v>
+        <v>0.158161447835326</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.0288792080868142</v>
+        <v>-0.0130572849002888</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0123637169981132</v>
+        <v>0.0121881449032149</v>
       </c>
       <c r="D10" t="n">
-        <v>-2.33580306725085</v>
+        <v>-1.07131027764895</v>
       </c>
       <c r="E10" t="n">
-        <v>0.020075592105186</v>
+        <v>0.284720775809009</v>
       </c>
     </row>
     <row r="11">
@@ -816,50 +816,50 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.032441084846519</v>
+        <v>0.0409257488241372</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0116300757079439</v>
+        <v>0.010910267356138</v>
       </c>
       <c r="D11" t="n">
-        <v>2.78941304091082</v>
+        <v>3.75112245082729</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00557440539491165</v>
+        <v>0.000203955563127836</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.0026221572434501</v>
+        <v>-0.00569374207398377</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0252974125142338</v>
+        <v>0.0222836186341765</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.10365317962755</v>
+        <v>-0.255512453675331</v>
       </c>
       <c r="E12" t="n">
-        <v>0.917504985883087</v>
+        <v>0.798467787629099</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.0120736553164605</v>
+        <v>-0.0120258168636827</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0127879449155814</v>
+        <v>0.0110427008350064</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.944143519241263</v>
+        <v>-1.08902858488747</v>
       </c>
       <c r="E13" t="n">
-        <v>0.345758948602271</v>
+        <v>0.276842504152492</v>
       </c>
     </row>
   </sheetData>
@@ -886,7 +886,7 @@
         <v>22</v>
       </c>
       <c r="B2" t="n">
-        <v>0.108299531732863</v>
+        <v>0.108838917946327</v>
       </c>
     </row>
     <row r="3">
@@ -894,7 +894,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="n">
-        <v>0.988634638678018</v>
+        <v>0.988492544513408</v>
       </c>
     </row>
     <row r="4">
@@ -902,7 +902,7 @@
         <v>24</v>
       </c>
       <c r="B4" t="n">
-        <v>0.988271211426443</v>
+        <v>0.988154089940273</v>
       </c>
     </row>
     <row r="5">
@@ -910,7 +910,7 @@
         <v>25</v>
       </c>
       <c r="B5" t="n">
-        <v>2720.30959261718</v>
+        <v>2920.60625849171</v>
       </c>
     </row>
     <row r="6">
@@ -926,7 +926,7 @@
         <v>27</v>
       </c>
       <c r="B7" t="n">
-        <v>344</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>